<commit_message>
Add Redis caching to v3, streaming visibility, and SQL grounding for NL2SQL answers
</commit_message>
<xml_diff>
--- a/Other_Documents/Progress plan.xlsx
+++ b/Other_Documents/Progress plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Nexus\Other_Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{601A06E3-B91C-4F66-BC9C-8ECB3ED81BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8C4081-0E31-4C5B-8914-7A594F7B2097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="39">
   <si>
     <t>Date</t>
   </si>
@@ -125,6 +125,48 @@
   </si>
   <si>
     <t>I agent pick info, which is wrong then agent reditect to human to review, update the vector - selfheal AI</t>
+  </si>
+  <si>
+    <t>Project scaffolding</t>
+  </si>
+  <si>
+    <t>Day 4</t>
+  </si>
+  <si>
+    <t>Day 5</t>
+  </si>
+  <si>
+    <t>Day 7</t>
+  </si>
+  <si>
+    <t>Day 8</t>
+  </si>
+  <si>
+    <t>Rag Implementation SOW</t>
+  </si>
+  <si>
+    <t>Rag - Eval Harness and Questions</t>
+  </si>
+  <si>
+    <t>Rag Implementation - DB Se up</t>
+  </si>
+  <si>
+    <t>Nl2SQL Implementation</t>
+  </si>
+  <si>
+    <t>Day 9</t>
+  </si>
+  <si>
+    <t>Day 10</t>
+  </si>
+  <si>
+    <t>RAG + NL2SQL Integration</t>
+  </si>
+  <si>
+    <t>Single agent vs Agentic Implementation</t>
+  </si>
+  <si>
+    <t>treat rag and NL2SQL as diff tool to treat as agentic ai vs single agent</t>
   </si>
 </sst>
 </file>
@@ -547,7 +589,7 @@
         <v>46288</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>12</v>
@@ -558,47 +600,120 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
+      <c r="B5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="2">
+        <f>C4+1</f>
+        <v>46289</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
+      <c r="B6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2">
+        <v>46289</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
+      <c r="B7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2">
+        <v>46290</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
+      <c r="B8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="2">
+        <v>46293</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
+      <c r="B9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="2">
+        <v>46294</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
+      <c r="B10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="2">
+        <v>46295</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
+      <c r="B11" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="2">
+        <v>46295</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <f t="shared" si="0"/>
         <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2">
+        <v>46302</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
implement Guardrails - Day 13
</commit_message>
<xml_diff>
--- a/Other_Documents/Progress plan.xlsx
+++ b/Other_Documents/Progress plan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Nexus\Other_Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26FE804B-95FD-4B97-9D2D-4A9276675610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2F66E79-BEF2-4249-938D-44FBD4B0B377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20400" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
   <si>
     <t>Date</t>
   </si>
@@ -198,6 +198,15 @@
   </si>
   <si>
     <t>Call Tavily tool in Nuxus</t>
+  </si>
+  <si>
+    <t>Day 13</t>
+  </si>
+  <si>
+    <t>Implement Guardrails</t>
+  </si>
+  <si>
+    <t>Guardrails at Direct prompt injection (input), Not use websearch as free llm (Input), Rag response groundedness (Output)</t>
   </si>
 </sst>
 </file>
@@ -812,6 +821,18 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
+      <c r="B16" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" s="2">
+        <v>46309</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>50</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>